<commit_message>
Removed scrolling offset from library preparation with selection template.
</commit_message>
<xml_diff>
--- a/backend/fms_core/static/submission_templates/Library_preparation_with_selection_v5_8_0.xlsx
+++ b/backend/fms_core/static/submission_templates/Library_preparation_with_selection_v5_8_0.xlsx
@@ -11691,7 +11691,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -11816,12 +11816,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="15">
@@ -11986,7 +11980,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -12184,10 +12178,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -42124,7 +42114,7 @@
       <c r="N19" s="14"/>
       <c r="O19" s="14"/>
       <c r="P19" s="14"/>
-      <c r="R19" s="50" t="s">
+      <c r="R19" s="24" t="s">
         <v>116</v>
       </c>
       <c r="S19" s="14"/>

</xml_diff>

<commit_message>
Fixes to the library preparation with selection template. Added Bacteriophage field as a property type to record it.
</commit_message>
<xml_diff>
--- a/backend/fms_core/static/submission_templates/Library_preparation_with_selection_v5_8_0.xlsx
+++ b/backend/fms_core/static/submission_templates/Library_preparation_with_selection_v5_8_0.xlsx
@@ -12373,9 +12373,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="1" width="15.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="31.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="38.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="31.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="44.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="18" style="1" width="15.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="22" style="1" width="10.43"/>
   </cols>
@@ -25777,11 +25777,11 @@
       <formula1>Index!$H$2:$H$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I7:L78 R7:R500 J79:L79 I80:L500" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J7:L500 R7:R500" type="none">
       <formula1>Index!$N$2:$N$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I79" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I7:I500" type="list">
       <formula1>Index!$G$2:$G$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -25980,7 +25980,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="22"/>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -25996,7 +25996,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="22"/>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -26012,7 +26012,7 @@
       <c r="Q7" s="3"/>
       <c r="R7" s="22"/>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -26028,7 +26028,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="22"/>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -26044,7 +26044,7 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="22"/>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -26060,7 +26060,7 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="22"/>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -26076,7 +26076,7 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="22"/>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -26092,7 +26092,7 @@
       <c r="Q12" s="3"/>
       <c r="R12" s="22"/>
     </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -26108,7 +26108,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="22"/>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -26124,7 +26124,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="22"/>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -26140,7 +26140,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="22"/>
     </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -26156,7 +26156,7 @@
       <c r="Q16" s="3"/>
       <c r="R16" s="22"/>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -26172,7 +26172,7 @@
       <c r="Q17" s="3"/>
       <c r="R17" s="22"/>
     </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -26188,7 +26188,7 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="22"/>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -26204,7 +26204,7 @@
       <c r="Q19" s="3"/>
       <c r="R19" s="22"/>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -38589,7 +38589,7 @@
       <c r="O1000" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M221:M384" type="list">
       <formula1>Index!$R$2:$R$20</formula1>
       <formula2>0</formula2>
@@ -38614,12 +38614,16 @@
       <formula1>Index!$J$18:$J$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="O5:O1000" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="O501:O1000" type="list">
       <formula1>INDIRECT(SUBSTITUTE(Q5," ","_"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="N5:N1000" type="list">
       <formula1>Index!$R$2:$R$31</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="O5:O500" type="list">
+      <formula1>INDIRECT(SUBSTITUTE(N5," ","_"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Added a test for library preparation with selection importer.
</commit_message>
<xml_diff>
--- a/backend/fms_core/static/submission_templates/Library_preparation_with_selection_v5_8_0.xlsx
+++ b/backend/fms_core/static/submission_templates/Library_preparation_with_selection_v5_8_0.xlsx
@@ -159,7 +159,7 @@
     <t xml:space="preserve">PCR Enzyme Lot</t>
   </si>
   <si>
-    <t xml:space="preserve">Library Preparation Template</t>
+    <t xml:space="preserve">Library Preparation with Selection Template</t>
   </si>
   <si>
     <t xml:space="preserve">Sample Information</t>
@@ -12365,7 +12365,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AE996"/>
-  <sheetFormatPr defaultColWidth="14.51171875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.14"/>
@@ -12392,7 +12392,7 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -25802,11 +25802,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB1000"/>
-  <sheetFormatPr defaultColWidth="14.51171875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="29.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="27.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="28.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20.29"/>
@@ -38643,7 +38643,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R84"/>
-  <sheetFormatPr defaultColWidth="9.17578125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.56"/>
   </cols>
@@ -39734,7 +39734,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AW1000"/>
-  <sheetFormatPr defaultColWidth="14.51171875" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="26.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="1" width="33.19"/>
@@ -39743,10 +39743,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="42.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="43.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="15.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="1" width="19.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="51.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="32.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="32.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="41.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="44.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="40.79"/>
@@ -39766,7 +39766,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="48.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="31.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="33.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="33.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="34.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="36.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="33.19"/>
@@ -39924,7 +39924,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="45" t="s">
         <v>129</v>
       </c>
@@ -40071,7 +40071,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="45" t="s">
         <v>169</v>
       </c>
@@ -40212,7 +40212,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="45" t="s">
         <v>207</v>
       </c>
@@ -40344,7 +40344,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="45" t="s">
         <v>242</v>
       </c>
@@ -40476,7 +40476,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="45" t="s">
         <v>276</v>
       </c>
@@ -40606,7 +40606,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="45" t="s">
         <v>309</v>
       </c>
@@ -40736,7 +40736,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="45" t="s">
         <v>342</v>
       </c>
@@ -40866,7 +40866,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="45" t="s">
         <v>374</v>
       </c>
@@ -41119,7 +41119,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="45" t="s">
         <v>437</v>
       </c>
@@ -41245,7 +41245,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="45" t="s">
         <v>470</v>
       </c>
@@ -41367,7 +41367,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="45" t="s">
         <v>500</v>
       </c>

</xml_diff>